<commit_message>
climate zones added to market template and adoption model output
now a new filter has been added to everything including the workpapers
</commit_message>
<xml_diff>
--- a/001_input/00_Master_Input_Template.xlsx
+++ b/001_input/00_Master_Input_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/Potential_Study_Tool_Prototype/001_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{FD06DD39-32B3-4C2A-BD0A-B82B14226CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91FA266D-A77D-4625-97E4-9B877137C441}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{FD06DD39-32B3-4C2A-BD0A-B82B14226CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF8D9DD2-C1F0-487B-BEE1-42EC4BFB0FAA}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1890" yWindow="3405" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="kwh_kw_ratio" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="121">
   <si>
     <t>parent_condition_name</t>
   </si>
@@ -408,6 +408,9 @@
   </si>
   <si>
     <t>refrigerator_electricity_existing_residential</t>
+  </si>
+  <si>
+    <t>climate_zone</t>
   </si>
 </sst>
 </file>
@@ -2300,17 +2303,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="15.140625" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -2318,101 +2321,113 @@
         <v>9</v>
       </c>
       <c r="C1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
         <v>50000</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>25000</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>5000</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
         <v>100000</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="1">
         <v>50000</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>20000</v>
       </c>
-      <c r="F3" s="1">
+      <c r="G3" s="1">
         <v>10000</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1">
         <v>275000</v>
       </c>
-      <c r="D4" s="1">
+      <c r="E4" s="1">
         <v>47000</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <v>19000</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="1">
         <v>7000</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C5" s="1"/>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C6" s="1"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C7" s="1"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C8" s="1"/>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
extensive PRD for Programs and phase 1 completed
</commit_message>
<xml_diff>
--- a/001_input/00_Master_Input_Template.xlsx
+++ b/001_input/00_Master_Input_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/Potential_Study_Tool_Prototype/001_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{FD06DD39-32B3-4C2A-BD0A-B82B14226CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCB5DEC8-322C-42D1-9F09-1376130C710E}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{FD06DD39-32B3-4C2A-BD0A-B82B14226CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60330927-7426-4B2C-A472-FDED8E86B499}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-3420" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-3420" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="kwh_kw_ratio" sheetId="1" r:id="rId1"/>
@@ -6256,7 +6256,9 @@
   <dimension ref="A1:D109"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
+    <col min="4" max="4" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>